<commit_message>
mdm logics are upgraded
</commit_message>
<xml_diff>
--- a/HMDM_DEV_Cleaned.xlsx
+++ b/HMDM_DEV_Cleaned.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="7" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Raw" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_to_Land" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Land_to_Stag" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stg_MDM_Ingress-HCP" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stg_MDM_Ingress-HCO" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MDM_HUB_Egress-HCP_Master" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MDM_HUB_Egress-HCO_Master" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HMDM_Physical_Inventory" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_Trail_Log" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Fixes_Applied_Log" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Tables" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Source_Raw" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Raw_to_Land" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Land_to_Stag" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Stg_MDM_Ingress-HCP" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Stg_MDM_Ingress-HCO" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MDM_HUB_Egress-HCP_Master" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MDM_HUB_Egress-HCO_Master" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="HMDM_Physical_Inventory" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Audit_Trail_Log" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Data_Fixes_Applied_Log" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tables'!$A$1:$C$25</definedName>
@@ -1184,7 +1184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1569,6 +1569,357 @@
       <c r="E14" s="28" t="inlineStr">
         <is>
           <t>All four corrected in earlier passes - see Data_Fixes_Applied_Log for exact before/after detail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>#20 Notebook 07 ingress batch fix</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07_MDM_Ingress / mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Batch status marked Y after first table, blocking remaining 12 tables</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Added skip_batch_update param; notebook resets/updates batch status post-loop</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>#21 Notebook 07 source table qualification</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Source tables not schema-qualified (hcp_name vs hmdm_dev.staging.hcp_name)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Auto-qualify with stg_schema from runtime_config</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>#22 Notebook 07 HCP field mapping mismatch</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>DEV_HCP_FIELD_MAPPING used camelCase, staging has snake_case</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Changed to snake_case: iqvia_id, first_name, middle_name, last_name, country_code</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>#23 Notebook 07 MDM target qualification</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Target table mdm.hcp missing catalog prefix (hmdm_dev.mdm.hcp)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Auto-qualify with catalog.publish_schema.physical_target</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>#24 Notebook 07 HCP child table mapping</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>All 13 HCP source tables written to single mdm.hcp, no child tables</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Added HCP_SOURCE_TO_MDM: hcp_name-&gt;hcp, hcp_specialty-&gt;hcp_specialty, hcp_identification-&gt;hcp_license, hcp_education-&gt;hcp_therapeutic_area</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>#25 Notebook 07 HCO ingress support</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>No HCO field mapping or HCO ingress logic existed</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Added DEV_HCO_FIELD_MAPPING, HCO_SOURCE_TO_MDM, prepare_hco_simple_ingress, process_hco_simple_ingress</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>#26 Notebook 07 table auto-create</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>write_prepared_ingress raised error if MDM target table didn't exist</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Removed pre-existence check; saveAsTable auto-creates on first run</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>#27 Notebook 08 egress batch fix</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08_MDM_Egress / mdm_egress.py</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Egress marked batch Y after first group, blocking remaining groups</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Added skip_batch_update param; notebook updates batch status post-loop</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>#28 Notebook 08 egress table auto-create</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>mdm_egress.py</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>write_egress raised error if MASTER target table didn't exist</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Removed pre-existence check; saveAsTable auto-creates on first run</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>#29 Notebook 08 widget default fix</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08_MDM_Egress</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Widget source_system_name defaulted to IQVIA, batch log has IQVIA_API</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Resolved - notebook cell fix</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Changed widget default to IQVIA_API in Cell 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>#30 runtime_config warning suppress</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>core/runtime_config.py</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Warning: Failed to extract job context printed on every Serverless run</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Resolved - code fix in .py</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Changed print to silent pass; JVM API not available on Spark Connect</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>#31 Notebook 07 Cell 12 cleanup</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07_MDM_Ingress</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Cell 12 had relative-import error handling masking real failures</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Resolved - notebook cell fix</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Simplified to raise RuntimeError on any failure; removed import-error workaround</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>#32 Notebook 07 Cell 10 env fix</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07_MDM_Ingress</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Cell 10 print had 'unknown' instead of {env} variable</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Resolved - notebook cell fix</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Restored to print(f'Environment : {env}')</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -1611,342 +1962,631 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="42" t="inlineStr">
+      <c r="A2" s="47" t="inlineStr">
         <is>
           <t>Source_Raw</t>
         </is>
       </c>
-      <c r="B2" s="42" t="inlineStr">
+      <c r="B2" s="47" t="inlineStr">
         <is>
           <t>Extra blank 7th column with no header/data</t>
         </is>
       </c>
-      <c r="C2" s="42" t="inlineStr">
+      <c r="C2" s="47" t="inlineStr">
         <is>
           <t>Removed the empty column</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="43" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>Raw_to_Land</t>
         </is>
       </c>
-      <c r="B3" s="43" t="inlineStr">
+      <c r="B3" s="48" t="inlineStr">
         <is>
           <t>17 rows (HCO_ADDRESS, HCO_ALTERNATE_NAME, HCO_EMAIL, HCO_HIERARCHY, HCO_IDENTIFICATION, HCO_NAME, HCO_PHONE, HCO_SPECIALTY, HCO_TAX, HCP_EDUCATION, HCP_EMAIL, HCP_HCO_AFFILIATION, HCP_LANGUAGE, HCP_ORIGIN_UNIVERSITY, HCP_PHONE, HCP_TAX, HCP_TENDENCIES) had "Pass Through" wrongly placed in the Source Column field, leaving Target Column blank</t>
         </is>
       </c>
-      <c r="C3" s="43" t="inlineStr">
+      <c r="C3" s="48" t="inlineStr">
         <is>
           <t>Corrected both Source Column and Target Column to read "All Columns (Pass Through)" to represent full-table pass-through mapping</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
         <is>
           <t>Land_to_Stag</t>
         </is>
       </c>
-      <c r="B4" s="42" t="inlineStr">
+      <c r="B4" s="47" t="inlineStr">
         <is>
           <t>Row 2: Src_tbl_nm listed as HMDM_DEV.LANDING.HCP_NAME but the DQ column (hco_name) and Target_tbl_nm (HMDM_DEV.STAGING.HCO_NAME) both point to HCO, not HCP</t>
         </is>
       </c>
-      <c r="C4" s="42" t="inlineStr">
+      <c r="C4" s="47" t="inlineStr">
         <is>
           <t>Corrected Src_tbl_nm to HMDM_DEV.LANDING.HCO_NAME</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="43" t="inlineStr">
+      <c r="A5" s="48" t="inlineStr">
         <is>
           <t>Land_to_Stag</t>
         </is>
       </c>
-      <c r="B5" s="43" t="inlineStr">
+      <c r="B5" s="48" t="inlineStr">
         <is>
           <t>Header 'mn_name/DQ_appl' was unclear / inconsistent naming</t>
         </is>
       </c>
-      <c r="C5" s="43" t="inlineStr">
+      <c r="C5" s="48" t="inlineStr">
         <is>
           <t>Renamed header to 'Column_Name'</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="42" t="inlineStr">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>Pending_Mappings_Tracker (new sheet)</t>
         </is>
       </c>
-      <c r="B6" s="42" t="inlineStr">
+      <c r="B6" s="47" t="inlineStr">
         <is>
           <t>Cross-checked HMDM_Physical_Inventory against the 4 mapping sheets to find STAGING/MDM tables with no corresponding ingress/egress mapping rows yet</t>
         </is>
       </c>
-      <c r="C6" s="42" t="inlineStr">
+      <c r="C6" s="47" t="inlineStr">
         <is>
           <t>Added a tracker sheet listing every gap found so mapping work can be completed</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="43" t="inlineStr">
+      <c r="A7" s="48" t="inlineStr">
         <is>
           <t>Tables</t>
         </is>
       </c>
-      <c r="B7" s="43" t="inlineStr">
+      <c r="B7" s="48" t="inlineStr">
         <is>
           <t>Table inventory was missing 4 entries even though full RAW/LANDING/STAGING lineage already exists for them elsewhere in the workbook: HCP_TAX, HCP_EMAIL, HCO_TAX, HCO_EMAIL</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C7" s="48" t="inlineStr">
         <is>
           <t>Added the 4 missing rows to the Tables sheet using the existing naming convention (raw_Healthcare_&lt;entity&gt; -&gt; HMDM_DEV.LANDING.&lt;TABLE&gt;), sourced directly from Source_Raw/Raw_to_Land/Land_to_Stag data already present in the workbook</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="42" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>Raw_to_Land</t>
         </is>
       </c>
-      <c r="B8" s="42" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Source Column for one HCP_IDENTIFICATION row was the literal "IQVIA ID'" with a stray trailing quote character</t>
         </is>
       </c>
-      <c r="C8" s="42" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Corrected to "IQVIA ID"</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="43" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>Pending_Mappings_Tracker (rebuilt)</t>
         </is>
       </c>
-      <c r="B9" s="43" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>Cross-checked all 8 supporting DOCX files (src_to_raw, raw_to_std_canonical, raw_to_land_std, download_api, IQVIA_API, log_file, start_file, common_functions) against every mapping sheet, and ran full referential-integrity checks across the RAW-&gt;LANDING-&gt;STAGING-&gt;MDM Ingress-&gt;MDM Egress chain</t>
         </is>
       </c>
-      <c r="C9" s="43" t="inlineStr">
+      <c r="C9" s="48" t="inlineStr">
         <is>
           <t>Rebuilt the tracker against the full 20-point checklist: confirmed gaps needing real source input, architecture patterns needing sign-off, and one duplicate-mapping and one HCP/HCO-block anomaly flagged for verification. Nothing was fabricated to fill these - see Recommended_Next_Step in each row</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="42" t="inlineStr">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>Source_Raw</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="47" t="inlineStr">
         <is>
           <t>HCP_ORIGIN_UNIVERSITY had zero RAW-level source mapping anywhere</t>
         </is>
       </c>
-      <c r="C10" s="42" t="inlineStr">
+      <c r="C10" s="47" t="inlineStr">
         <is>
           <t>Added a proposed IQVIA JSON path (individual.OriginUniversity[*].universityName/universityCode/graduationYear), orange-highlighted as NOT confirmed - needs validation against the real API contract</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="A11" s="48" t="inlineStr">
         <is>
           <t>Raw_to_Land</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
         <is>
           <t>17 tables only said "All Columns (Pass Through)" with no field-level detail</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="48" t="inlineStr">
         <is>
           <t>Expanded each into Source_FK + MD5 surrogate PK + every real RAW column (from Source_Raw) + standard Source_Name/Source_Created_Date/Source_Updated_Date audit columns, following the exact pattern already used by HCP_NAME/HCP_ADDRESS/HCP_SPECIALTY etc. in this same workbook. Green-highlighted as newly authored this round</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="42" t="inlineStr">
+      <c r="A12" s="47" t="inlineStr">
         <is>
           <t>Stg_MDM_Ingress-HCP</t>
         </is>
       </c>
-      <c r="B12" s="42" t="inlineStr">
+      <c r="B12" s="47" t="inlineStr">
         <is>
           <t>HCP_HCO_AFFILIATION, HCP_LANGUAGE, HCP_ORIGIN_UNIVERSITY, HCP_TENDENCIES had full upstream lineage but no MDM ingress mapping</t>
         </is>
       </c>
-      <c r="C12" s="42" t="inlineStr">
+      <c r="C12" s="47" t="inlineStr">
         <is>
           <t>Added 7 rows into MDM.HCP using the existing X_infac360ls_/X_* naming convention. Green-highlighted - proposed target attribute names, please validate against the real Informatica base-object config</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>Stg_MDM_Ingress-HCO</t>
         </is>
       </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="B13" s="48" t="inlineStr">
         <is>
           <t>HCO_ADDRESS, HCO_ALTERNATE_NAME, HCO_EMAIL, HCO_HIERARCHY, HCO_TAX had full upstream lineage but no MDM ingress mapping</t>
         </is>
       </c>
-      <c r="C13" s="43" t="inlineStr">
+      <c r="C13" s="48" t="inlineStr">
         <is>
           <t>Added 10 rows, consolidated onto core MDM.HCO (mirroring how HCP consolidates address/phone/email/tax onto core MDM.HCP). Green-highlighted - please validate</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="42" t="inlineStr">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>MDM_HUB_Egress-HCP_Master</t>
         </is>
       </c>
-      <c r="B14" s="42" t="inlineStr">
+      <c r="B14" s="47" t="inlineStr">
         <is>
           <t>Core MDM.HCP object had no egress/master mapping at all</t>
         </is>
       </c>
-      <c r="C14" s="42" t="inlineStr">
+      <c r="C14" s="47" t="inlineStr">
         <is>
           <t>Added a 23-attribute core egress block as pass-through exposure. Green-highlighted - please validate whether business-friendly renaming (like the existing Specialty block) is expected instead</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="43" t="inlineStr">
+      <c r="A15" s="48" t="inlineStr">
         <is>
           <t>MDM_HUB_Egress-HCO_Master</t>
         </is>
       </c>
-      <c r="B15" s="43" t="inlineStr">
+      <c r="B15" s="48" t="inlineStr">
         <is>
           <t>Core MDM.HCO object had no egress/master mapping at all</t>
         </is>
       </c>
-      <c r="C15" s="43" t="inlineStr">
+      <c r="C15" s="48" t="inlineStr">
         <is>
           <t>Added a 10-attribute core egress block (only the newly-added attributes) as pass-through, consistent with the rest of this sheet. Green-highlighted</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="42" t="inlineStr">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>Stg_MDM_Ingress-HCO - HCO_NAME</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="47" t="inlineStr">
         <is>
           <t>18 of 26 STAGING.HCO_NAME attributes (Bed_Count, Teaching_Hospital_Flag, Accept_Medicare, etc.) have no RAW/LANDING source anywhere in this workbook or the 8 DOCX files</t>
         </is>
       </c>
-      <c r="C16" s="42" t="inlineStr">
+      <c r="C16" s="47" t="inlineStr">
         <is>
           <t>Deliberately NOT fabricated - flagged in Pending_Mappings_Tracker as a critical open item, since inventing a fake source for real hospital-facility data would violate the "no fake source fields" rule. Needs your input on the real upstream feed</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="43" t="inlineStr">
+      <c r="A17" s="48" t="inlineStr">
         <is>
           <t>MDM_HUB_Egress-HCP_Master</t>
         </is>
       </c>
-      <c r="B17" s="43" t="inlineStr">
+      <c r="B17" s="48" t="inlineStr">
         <is>
           <t>Re-verified per your request: the core-HCP block added last round used plain passthrough naming, inconsistent with every existing HCP egress block (which all rename X_infa360_*/X_infac360ls_* system attributes to business-friendly names)</t>
         </is>
       </c>
-      <c r="C17" s="43" t="inlineStr">
+      <c r="C17" s="48" t="inlineStr">
         <is>
           <t>Replaced with 23 properly renamed rows (First_Name, Last_Name, DEA_Number, Language, Tendency_Code, etc.), matching the established convention exactly</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="42" t="inlineStr">
+      <c r="A18" s="47" t="inlineStr">
         <is>
           <t>MDM_HUB_Egress-HCO_Master</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B18" s="47" t="inlineStr">
         <is>
           <t>Re-verified per your request: cross-checked all 4 existing HCO egress blocks</t>
         </is>
       </c>
-      <c r="C18" s="42" t="inlineStr">
+      <c r="C18" s="47" t="inlineStr">
         <is>
           <t>Confirmed pure passthrough (no renaming) is the correct, consistent, already-established pattern for HCO - the new core-HCO block correctly matches it, no change needed</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="43" t="inlineStr">
+      <c r="A19" s="48" t="inlineStr">
         <is>
           <t>Source_Raw + Raw_to_Land - HCO_NAME</t>
         </is>
       </c>
-      <c r="B19" s="43" t="inlineStr">
+      <c r="B19" s="48" t="inlineStr">
         <is>
           <t>The 18 STAGING.HCO_NAME facility-profile attributes with no source anywhere were the one item deliberately left open last round</t>
         </is>
       </c>
-      <c r="C19" s="43" t="inlineStr">
+      <c r="C19" s="48" t="inlineStr">
         <is>
           <t>Per your instruction to fill remaining pending items using realtime project flow where DOCX has no answer, added a proposed organization.facilityProfile.*/organization.* JSON structure covering all 18 attributes. Orange-highlighted as proposed/needs validation - NOT confirmed against a real IQVIA schema</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="42" t="inlineStr">
+      <c r="A20" s="47" t="inlineStr">
         <is>
           <t>Land_to_Stag - HCP_LICENSE</t>
         </is>
       </c>
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B20" s="47" t="inlineStr">
         <is>
           <t>Left undocumented last round pending your confirmation</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C20" s="47" t="inlineStr">
         <is>
           <t>Added an explicit row documenting that HCP_LICENSE is sourced via the separate real-time IQVIA&lt;-&gt;Kokoro Lambda integration described in download_api.docx, so nothing is left as a silent/blank gap</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="43" t="inlineStr">
+      <c r="A21" s="48" t="inlineStr">
         <is>
           <t>Audit_Trail_Log (renamed from Pending_Mappings_Tracker)</t>
         </is>
       </c>
-      <c r="B21" s="43" t="inlineStr">
+      <c r="B21" s="48" t="inlineStr">
         <is>
           <t>Every previously-open item has now been actioned</t>
         </is>
       </c>
-      <c r="C21" s="43" t="inlineStr">
+      <c r="C21" s="48" t="inlineStr">
         <is>
           <t>All 13 tracked items are now Resolved or Proposed-needs-validation - nothing is left marked as an unactioned gap. Proposed items are still clearly flagged (orange rows + Status column) since their real-world source could not be confirmed from the DOCX files, per your instruction to keep this traceable</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>All 13 HCP tables written to single mdm.hcp; no child tables created</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Added HCP_SOURCE_TO_MDM mapping (13 entries) + DEV_HCO_FIELD_MAPPING + HCO_SOURCE_TO_MDM (9 entries)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Batch status set to Y after first table in process_ingress</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Added skip_batch_update param to process_ingress() and main(); wrapped update_batch_log_tbl call</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Source tables not schema-qualified</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Auto-qualify source_table with stg_schema if not already qualified</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DEV_HCP_FIELD_MAPPING used camelCase columns not in staging</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Changed to snake_case: iqvia_id, first_name, middle_name, last_name, country_code</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MDM target table not catalog-qualified</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Auto-qualify with f'{_catalog}.{publish_schema}.{physical_target}'</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Table existence check blocked first-run ingress</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Removed _table_exists check; saveAsTable auto-creates</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>No HCO ingress support</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Added prepare_hco_simple_ingress(), process_hco_simple_ingress(), DEV_HCO_FIELD_MAPPING</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>mdm_ingress.py</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>process_ingress hardcoded target_table=hcp for all HCP</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Uses HCP_SOURCE_TO_MDM/HCO_SOURCE_TO_MDM lookup; supports one-to-many (hco_name-&gt;[hco,hco_name])</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>mdm_egress.py</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Egress marked batch Y after first group</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Added skip_batch_update param to process_egress_batch() and main_pipeline()</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>mdm_egress.py</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Table existence check blocked first-run egress</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Removed _table_exists check; saveAsTable auto-creates</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>runtime_config.py</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Warning printed on every Serverless run</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Silent pass instead of print() for JVM context extraction failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07_MDM_Ingress Cell 3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Widget default IQVIA instead of IQVIA_API</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Changed to IQVIA_API</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07_MDM_Ingress Cell 10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Missing skip_batch_update, no reset/update batch logic</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Added skip_batch_update=True, reset ingress_status=N, post-loop update to Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07_MDM_Ingress Cell 10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>print(f'Environment : unknown') hardcoded</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Restored to print(f'Environment : {env}')</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>07_MDM_Ingress Cell 12</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Relative-import error handling masked real failures</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Simplified to raise RuntimeError on any failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08_MDM_Egress Cell 3</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Widget default IQVIA instead of IQVIA_API</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Changed to IQVIA_API</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08_MDM_Egress Cell 10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Missing skip_batch_update, no table existence check, no reset/update</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Added skip_batch_update=True, spark.catalog.tableExists() skip, reset egress_status=N, post-loop update to Y</t>
         </is>
       </c>
     </row>
@@ -19889,7 +20529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -21978,6 +22618,600 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>HCP_ADDRESS</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCP_ADDRESS</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>HCP_PHONE</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCP_PHONE</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>HCP_EMAIL</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCP_EMAIL</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>HCP_TENDENCIES</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCP_TENDENCIES</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>HCP_ORIGIN_UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCP_ORIGIN_UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>HCP_TAX</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCP_TAX</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>HCP_LANGUAGE</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCP_LANGUAGE</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>HCP_HCO_AFFILIATION</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCP_HCO_AFFILIATION</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>HCO_ADDRESS</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCO_ADDRESS</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>HCO_EMAIL</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCO_EMAIL</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>HCO_IDENTIFICATION</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCO_IDENTIFICATION</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>HCO_HCO_HIERARCHY</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCO_HCO_HIERARCHY</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>MDM</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>HCO_TAX</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MDM.HCO_TAX</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Stg_MDM_Ingress (extra)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>HCP_SPECIALTY</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCP_SPECIALTY</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCP_Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HCP_ALTERNATE_NAME</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCP_ALTERNATE_NAME</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCP_Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>HCP_THERAPEUTIC_AREA</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCP_THERAPEUTIC_AREA</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCP_Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>HCP_LICENSE</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCP_LICENSE</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCP_Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>HCO</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCO</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCO_Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>HCO_NAME</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCO_NAME</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCO_Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>HCO_ALTERNATE_IDENTIFIER</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCO_ALTERNATE_IDENTIFIER</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCO_Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>HCO_PHONE</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCO_PHONE</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCO_Master</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>HCO_SPECIALTY</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>HMDM_DEV.MASTER.HCO_SPECIALTY</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>HMDM_DEV</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>MDM_HUB_Egress-HCO_Master</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>